<commit_message>
various changes to help with replicability and sharing
</commit_message>
<xml_diff>
--- a/report/scenario summary.xlsx
+++ b/report/scenario summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthiasfripp/Library/CloudStorage/OneDrive-EnergyInnovation/Analysis/Electricity-Shared/Load-Growth/Switch-USA-PG-ReEDS/report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energyinnovation.sharepoint.com/sites/Policy-Electricity/Shared Documents/Electricity/Load-Growth/Switch-USA-PG-ReEDS/report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08302C1-9E79-7A4A-9890-7F754FE9E842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="14_{8F24C7B9-61BD-DB49-BF82-5A0C9A926DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B239797-DF06-0442-881A-CAC32F1B07B3}"/>
   <bookViews>
-    <workbookView xWindow="11680" yWindow="760" windowWidth="22880" windowHeight="19880" xr2:uid="{023A4B6C-4A08-E24A-8297-A440EACD546C}"/>
+    <workbookView xWindow="18660" yWindow="760" windowWidth="22880" windowHeight="19880" xr2:uid="{023A4B6C-4A08-E24A-8297-A440EACD546C}"/>
   </bookViews>
   <sheets>
     <sheet name="cost vs emissions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>scenario</t>
   </si>
@@ -90,12 +90,6 @@
     <t>clean growth share</t>
   </si>
   <si>
-    <t>clean_400</t>
-  </si>
-  <si>
-    <t>clean_500</t>
-  </si>
-  <si>
     <t>expected</t>
   </si>
   <si>
@@ -106,9 +100,6 @@
   </si>
   <si>
     <t>diff from base</t>
-  </si>
-  <si>
-    <t>for f in out/{2025,2030/ce}/*/total_cost.txt; do dir=${f:h}; q "select split_part('$dir', '/', -1) as case, * from (select period, sum(DispatchEmissions_tCO2_per_typical_yr/1e9) as GtCO2, sum(Energy_GWh_typical_yr*0.001) filter (DispatchEmissions_tCO2_per_typical_yr = 0 and gen_energy_source not in ('imports', 'storage')) as clean_TWh, sum(Energy_GWh_typical_yr*0.001) filter (DispatchEmissions_tCO2_per_typical_yr &gt; 0 and gen_energy_source not in ('imports', 'storage')) as dirty_TWh from '$dir/dispatch_annual_summary.csv' group by 1), (select (total_cost/1e9)*1.03**(2030-2025) as total_cost_B from read_csv('$dir/total_cost.txt', header=false, columns={'total_cost': 'DOUBLE'}))" | tail -n 1; done</t>
   </si>
   <si>
     <t>GtCO2</t>
@@ -150,9 +141,6 @@
     <t>label</t>
   </si>
   <si>
-    <t>dir=out/2030/ce/clean; q "select period, sum(DeployEEGWh_per_year) * 0.001 as ee_TWh from '$dir/energy_efficiency_investment.csv' group by 1"</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -179,6 +167,15 @@
   <si>
     <t>diff w/$200 SCC</t>
   </si>
+  <si>
+    <t>for f in out/{2025,2030/ce}/*/total_cost.txt; do dir=${f:h}; python report/q.py "select split_part('$dir', '/', -1) as case, * from (select period, sum(DispatchEmissions_tCO2_per_typical_yr/1e9) as GtCO2, sum(Energy_GWh_typical_yr*0.001) filter (DispatchEmissions_tCO2_per_typical_yr = 0 and gen_energy_source not in ('imports', 'storage')) as clean_TWh, sum(Energy_GWh_typical_yr*0.001) filter (DispatchEmissions_tCO2_per_typical_yr &gt; 0 and gen_energy_source not in ('imports', 'storage')) as dirty_TWh from '$dir/dispatch_annual_summary.csv' group by 1), (select (total_cost/1e9)*1.03**(2030-2025) as total_cost_B from read_csv('$dir/total_cost.txt', header=false, columns={'total_cost': 'DOUBLE'}))" | tail -n 1; done</t>
+  </si>
+  <si>
+    <t>dir=out/2030/ce/clean; python report/q.py "select period, sum(DeployEEGWh_per_year) * 0.001 as ee_TWh from '$dir/energy_efficiency_investment.csv' group by 1"</t>
+  </si>
+  <si>
+    <t>data query:</t>
+  </si>
 </sst>
 </file>
 
@@ -190,7 +187,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -209,6 +206,19 @@
       <color rgb="FF0070C0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -232,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -242,6 +252,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -303,7 +315,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$7</c:f>
+              <c:f>'cost vs emissions'!$A$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -342,7 +354,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D9C6E72B-AE62-954B-8EC8-187186B01408}" type="CELLRANGE">
+                    <a:fld id="{BF98B907-CBC6-C047-942B-440A6DA260A3}" type="CELLRANGE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -352,7 +364,7 @@
                       <a:t>
 </a:t>
                     </a:r>
-                    <a:fld id="{D89CF00B-2C5D-6F41-B5AC-DEB6DFAA1F02}" type="YVALUE">
+                    <a:fld id="{80ED00DA-FEBA-8141-B13E-12795B73C241}" type="YVALUE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[Y VALUE]</a:t>
@@ -387,7 +399,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F6948E7E-F0F8-214E-BC53-236630821DF4}" type="CELLRANGE">
+                    <a:fld id="{E0B2D045-96EE-EB43-A77D-2575C9B8718B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -397,7 +409,7 @@
                       <a:t>
 </a:t>
                     </a:r>
-                    <a:fld id="{F6CDDB97-22EE-FA48-B62E-DC988C0746DE}" type="YVALUE">
+                    <a:fld id="{155FA133-700C-1B42-80EF-D7B46A7389F6}" type="YVALUE">
                       <a:rPr lang="en-US" baseline="0"/>
                       <a:pPr/>
                       <a:t>[Y VALUE]</a:t>
@@ -423,66 +435,6 @@
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-2D00-9546-B362-9AC648E0D37F}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000001-12C9-2648-9AA5-6DBAB32288A6}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000002-12C9-2648-9AA5-6DBAB32288A6}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -532,42 +484,30 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$7:$D$10</c:f>
+              <c:f>'cost vs emissions'!$D$5:$D$6</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.8811821233644299</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.1311641095226399</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$G$7:$G$10</c:f>
+              <c:f>'cost vs emissions'!$G$5:$G$6</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>70.250764043747012</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>56.772947892443028</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -576,20 +516,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -722,92 +656,6 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{D1E707A0-2F60-8245-9663-577A2445742E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{F16CB903-AD83-5A45-B284-BB899C557222}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{0000000C-2D00-9546-B362-9AC648E0D37F}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{D5EC805C-81B1-8D40-9FBA-D396676A1C4E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{0796D8D5-7F59-9546-A003-01479784F546}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000013-2D00-9546-B362-9AC648E0D37F}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -854,42 +702,30 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$3:$D$6</c:f>
+              <c:f>'cost vs emissions'!$D$3:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.84284793310867</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.13069976554854</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$G$3:$G$6</c:f>
+              <c:f>'cost vs emissions'!$G$3:$G$4</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>29.705229425086003</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>24.645689469813021</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -898,20 +734,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -926,7 +756,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$11</c:f>
+              <c:f>'cost vs emissions'!$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1050,66 +880,6 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000005-12C9-2648-9AA5-6DBAB32288A6}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000006-12C9-2648-9AA5-6DBAB32288A6}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1156,42 +926,30 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$11:$D$14</c:f>
+              <c:f>'cost vs emissions'!$D$7:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.58309575582479</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.92198577445123198</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$G$11:$G$14</c:f>
+              <c:f>'cost vs emissions'!$G$7:$G$8</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>7.8543927114540111</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>5.2274474399100086</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1200,20 +958,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -1615,7 +1367,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$7</c:f>
+              <c:f>'cost vs emissions'!$A$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1751,92 +1503,6 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{A718ACAE-FA2E-9F4B-BFF7-4AC87BC7146C}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{BF0C2FD2-EC43-4640-97F4-1261B2908C39}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000013-5CBD-3847-A90D-07E7B03B8167}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{31ED1552-A641-364E-A040-3AD339F4925F}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{E6653BA9-1035-494E-8811-CB9EF93D9626}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000014-5CBD-3847-A90D-07E7B03B8167}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1883,31 +1549,25 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$F$7:$F$10</c:f>
+              <c:f>'cost vs emissions'!$F$5:$F$6</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>0.38703453823810741</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.6089671398070815</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$G$7:$G$14</c:f>
+              <c:f>'cost vs emissions'!$G$5:$G$8</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>70.250764043747012</c:v>
                 </c:pt>
@@ -1915,22 +1575,10 @@
                   <c:v>56.772947892443028</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#N/A</c:v>
+                  <c:v>7.8543927114540111</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.8543927114540111</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>5.2274474399100086</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1939,20 +1587,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -2091,92 +1733,6 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{30328E9E-5ECB-914D-897C-9BCB6D3692F4}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{CBAD1C37-D174-C542-B6D5-C626F7BA7907}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000002-5CBD-3847-A90D-07E7B03B8167}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{43AA73B1-60C3-4F4C-8256-3A7F4C22DDFB}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US" baseline="0"/>
-                  </a:p>
-                  <a:p>
-                    <a:fld id="{A4D51C71-5EC0-424B-A78F-40381ED3EC4C}" type="YVALUE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[Y VALUE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000003-5CBD-3847-A90D-07E7B03B8167}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2223,31 +1779,25 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$F$3:$F$6</c:f>
+              <c:f>'cost vs emissions'!$F$3:$F$4</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>0.38643693040768434</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.6014004180371062</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>('cost vs emissions'!$G$3:$G$6,'cost vs emissions'!$G$11:$G$14)</c:f>
+              <c:f>('cost vs emissions'!$G$3:$G$4,'cost vs emissions'!$G$7:$G$8)</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>29.705229425086003</c:v>
                 </c:pt>
@@ -2255,22 +1805,10 @@
                   <c:v>24.645689469813021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>#N/A</c:v>
+                  <c:v>7.8543927114540111</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.8543927114540111</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>5.2274474399100086</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2279,20 +1817,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -2307,7 +1839,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$11</c:f>
+              <c:f>'cost vs emissions'!$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2431,66 +1963,6 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
-            <c:dLbl>
-              <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000004-5A9C-EE46-AF3F-A76C421A4CE8}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:dLblPos val="t"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:separator>
-</c:separator>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000005-5A9C-EE46-AF3F-A76C421A4CE8}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2537,42 +2009,30 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$F$11:$F$14</c:f>
+              <c:f>'cost vs emissions'!$F$7:$F$8</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.066043267390884</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>4.3768768088682908</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$G$11:$G$14</c:f>
+              <c:f>'cost vs emissions'!$G$7:$G$8</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.0" B/y"</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>7.8543927114540111</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>5.2274474399100086</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2581,20 +2041,14 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>'cost vs emissions'!$B$3:$B$6</c15:f>
+                <c15:f>'cost vs emissions'!$B$3:$B$4</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="4"/>
+                  <c:ptCount val="2"/>
                   <c:pt idx="0">
                     <c:v>High Fossil</c:v>
                   </c:pt>
                   <c:pt idx="1">
                     <c:v>Clean</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Clean 400</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Clean 500</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -3027,42 +2481,30 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$3:$D$6</c:f>
+              <c:f>'cost vs emissions'!$D$3:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.84284793310867</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.13069976554854</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$H$3:$H$6</c:f>
+              <c:f>'cost vs emissions'!$H$3:$H$4</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>88.09113800004198</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-59.398035467257003</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3079,7 +2521,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$7</c:f>
+              <c:f>'cost vs emissions'!$A$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3112,42 +2554,30 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$7:$D$10</c:f>
+              <c:f>'cost vs emissions'!$D$5:$D$6</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.8811821233644299</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.1311641095226399</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$H$7:$H$10</c:f>
+              <c:f>'cost vs emissions'!$H$5:$H$6</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>136.30351066985497</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-27.177908249807018</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3164,7 +2594,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'cost vs emissions'!$A$11</c:f>
+              <c:f>'cost vs emissions'!$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3197,42 +2627,30 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$D$11:$D$14</c:f>
+              <c:f>'cost vs emissions'!$D$7:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>1.58309575582479</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.92198577445123198</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'cost vs emissions'!$H$11:$H$14</c:f>
+              <c:f>'cost vs emissions'!$H$7:$H$8</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>14.289865829633991</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-120.55907571662162</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>#N/A</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5287,13 +4705,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>357909</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>127003</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>85439</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5325,13 +4743,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>392543</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>69272</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>792385</xdr:colOff>
-      <xdr:row>62</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>27709</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5924,7 +5342,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F7718AE-BB94-6E44-8D91-8B7316D18574}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="18.6640625" customWidth="1"/>
@@ -5939,10 +5357,10 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -5957,22 +5375,28 @@
         <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="L1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="R1" t="s">
-        <v>30</v>
+      <c r="R1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
@@ -5984,18 +5408,18 @@
         <v>S20X1</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2">
-        <f t="shared" ref="D2:D14" si="0">VLOOKUP($C2, $L$3:$O$34, 3, FALSE)</f>
+        <f t="shared" ref="D2:D8" si="0">VLOOKUP($C2, $L$3:$O$34, 3, FALSE)</f>
         <v>1.5509183902338901</v>
       </c>
       <c r="E2" s="2">
-        <f t="shared" ref="E2:E14" si="1">VLOOKUP($C2, $L$3:$R$34, 6, FALSE)</f>
+        <f t="shared" ref="E2:E8" si="1">VLOOKUP($C2, $L$3:$R$34, 6, FALSE)</f>
         <v>167.40612537004299</v>
       </c>
       <c r="F2" s="3" cm="1">
-        <f t="array" ref="F2:F16">VLOOKUP($C2:$C16, $L$3:$S$33, 8, FALSE)</f>
+        <f t="array" ref="F2:F10">VLOOKUP($C2:$C10, $L$3:$S$33, 8, FALSE)</f>
         <v>0</v>
       </c>
       <c r="G2" s="5">
@@ -6009,25 +5433,25 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="L2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" t="s">
         <v>18</v>
       </c>
-      <c r="M2" t="s">
+      <c r="P2" t="s">
         <v>19</v>
       </c>
-      <c r="N2" t="s">
+      <c r="Q2" t="s">
         <v>17</v>
       </c>
-      <c r="O2" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>20</v>
-      </c>
       <c r="R2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="S2" t="s">
         <v>9</v>
@@ -6035,10 +5459,10 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B14" si="2">PROPER(SUBSTITUTE(C3, "_", " "))</f>
+        <f t="shared" ref="B3:B8" si="2">PROPER(SUBSTITUTE(C3, "_", " "))</f>
         <v>High Fossil</v>
       </c>
       <c r="C3" t="s">
@@ -6060,13 +5484,13 @@
         <v>29.705229425086003</v>
       </c>
       <c r="H3" s="2">
-        <f t="shared" ref="H3:H14" si="4">G3+200*(D3-D$2)</f>
+        <f t="shared" ref="H3:H8" si="4">G3+200*(D3-D$2)</f>
         <v>88.09113800004198</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="L3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M3">
         <v>2025</v>
@@ -6086,14 +5510,14 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="2"/>
         <v>Clean</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="0"/>
@@ -6107,7 +5531,7 @@
         <v>1.6014004180371062</v>
       </c>
       <c r="G4" s="5">
-        <f t="shared" ref="G4:G14" si="5">E4-E$2</f>
+        <f t="shared" ref="G4:G8" si="5">E4-E$2</f>
         <v>24.645689469813021</v>
       </c>
       <c r="H4" s="2">
@@ -6120,7 +5544,7 @@
       </c>
       <c r="J4" s="2"/>
       <c r="L4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="M4">
         <v>2030</v>
@@ -6147,38 +5571,39 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="2"/>
-        <v>Clean 400</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2" t="e">
+        <v>Peak Fuel High Fossil</v>
+      </c>
+      <c r="C5" t="str" cm="1">
+        <f t="array" ref="C5:C6">"peak_fuel_"&amp;C3:C4</f>
+        <v>peak_fuel_high_fossil</v>
+      </c>
+      <c r="D5" s="2">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E5" s="2" t="e">
+        <v>1.8811821233644299</v>
+      </c>
+      <c r="E5" s="2">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F5" s="3" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="G5" s="5" t="e">
+        <v>237.65688941379</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0.38703453823810741</v>
+      </c>
+      <c r="G5" s="5">
         <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H5" s="2" t="e">
+        <v>70.250764043747012</v>
+      </c>
+      <c r="H5" s="2">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
+        <v>136.30351066985497</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="L5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M5">
         <v>2030</v>
@@ -6202,35 +5627,38 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="2"/>
-        <v>Clean 500</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2" t="e">
+        <v>Peak Fuel Clean</v>
+      </c>
+      <c r="C6" t="str">
+        <v>peak_fuel_clean</v>
+      </c>
+      <c r="D6" s="2">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E6" s="2" t="e">
+        <v>1.1311641095226399</v>
+      </c>
+      <c r="E6" s="2">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F6" s="3" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="G6" s="5" t="e">
+        <v>224.17907326248601</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1.6089671398070815</v>
+      </c>
+      <c r="G6" s="5">
         <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H6" s="2" t="e">
+        <v>56.772947892443028</v>
+      </c>
+      <c r="H6" s="2">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I6" s="2"/>
+        <v>-27.177908249807018</v>
+      </c>
+      <c r="I6" s="2">
+        <f>G5-G6</f>
+        <v>13.477816151303983</v>
+      </c>
       <c r="J6" s="2"/>
       <c r="L6" t="s">
         <v>2</v>
@@ -6257,34 +5685,34 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="2"/>
-        <v>Peak Fuel High Fossil</v>
+        <v>Low Growth High Fossil</v>
       </c>
       <c r="C7" t="str" cm="1">
-        <f t="array" ref="C7:C10">"peak_fuel_"&amp;C3:C6</f>
-        <v>peak_fuel_high_fossil</v>
+        <f t="array" ref="C7:C8">"low_growth_"&amp;C3:C4</f>
+        <v>low_growth_high_fossil</v>
       </c>
       <c r="D7" s="2">
         <f t="shared" si="0"/>
-        <v>1.8811821233644299</v>
+        <v>1.58309575582479</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="1"/>
-        <v>237.65688941379</v>
+        <v>175.260518081497</v>
       </c>
       <c r="F7" s="3">
-        <v>0.38703453823810741</v>
+        <v>1.066043267390884</v>
       </c>
       <c r="G7" s="5">
         <f t="shared" si="5"/>
-        <v>70.250764043747012</v>
+        <v>7.8543927114540111</v>
       </c>
       <c r="H7" s="2">
         <f t="shared" si="4"/>
-        <v>136.30351066985497</v>
+        <v>14.289865829633991</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -6313,41 +5741,41 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="2"/>
-        <v>Peak Fuel Clean</v>
+        <v>Low Growth Clean</v>
       </c>
       <c r="C8" t="str">
-        <v>peak_fuel_clean</v>
+        <v>low_growth_clean</v>
       </c>
       <c r="D8" s="2">
         <f t="shared" si="0"/>
-        <v>1.1311641095226399</v>
+        <v>0.92198577445123198</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="1"/>
-        <v>224.17907326248601</v>
+        <v>172.63357280995299</v>
       </c>
       <c r="F8" s="3">
-        <v>1.6089671398070815</v>
+        <v>4.3768768088682908</v>
       </c>
       <c r="G8" s="5">
         <f t="shared" si="5"/>
-        <v>56.772947892443028</v>
+        <v>5.2274474399100086</v>
       </c>
       <c r="H8" s="2">
         <f t="shared" si="4"/>
-        <v>-27.177908249807018</v>
+        <v>-120.55907571662162</v>
       </c>
       <c r="I8" s="2">
         <f>G7-G8</f>
-        <v>13.477816151303983</v>
+        <v>2.6269452715440025</v>
       </c>
       <c r="J8" s="2"/>
       <c r="L8" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="M8">
         <v>2030</v>
@@ -6374,36 +5802,11 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="2"/>
-        <v>Peak Fuel Clean 400</v>
-      </c>
-      <c r="C9" t="str">
-        <v>peak_fuel_clean_400</v>
-      </c>
-      <c r="D9" s="2" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E9" s="2" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
       <c r="F9" s="3" t="e">
         <v>#N/A</v>
       </c>
-      <c r="G9" s="5" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H9" s="2" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="L9" t="s">
         <v>6</v>
@@ -6429,39 +5832,14 @@
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="2"/>
-        <v>Peak Fuel Clean 500</v>
-      </c>
-      <c r="C10" t="str">
-        <v>peak_fuel_clean_500</v>
-      </c>
-      <c r="D10" s="2" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E10" s="2" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
       <c r="F10" s="3" t="e">
         <v>#N/A</v>
       </c>
-      <c r="G10" s="5" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H10" s="2" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="L10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="M10">
         <v>2030</v>
@@ -6488,37 +5866,16 @@
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="2"/>
-        <v>Low Growth High Fossil</v>
-      </c>
-      <c r="C11" t="str" cm="1">
-        <f t="array" ref="C11:C14">"low_growth_"&amp;C3:C6</f>
-        <v>low_growth_high_fossil</v>
-      </c>
-      <c r="D11" s="2">
-        <f t="shared" si="0"/>
-        <v>1.58309575582479</v>
-      </c>
-      <c r="E11" s="2">
-        <f t="shared" si="1"/>
-        <v>175.260518081497</v>
-      </c>
-      <c r="F11" s="3">
-        <v>1.066043267390884</v>
-      </c>
-      <c r="G11" s="5">
-        <f t="shared" si="5"/>
-        <v>7.8543927114540111</v>
-      </c>
-      <c r="H11" s="2">
-        <f t="shared" si="4"/>
-        <v>14.289865829633991</v>
-      </c>
-      <c r="I11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
+      <c r="H11" t="s">
+        <v>29</v>
+      </c>
+      <c r="I11" s="5">
+        <f>G3</f>
+        <v>29.705229425086003</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="L11" t="s">
         <v>4</v>
@@ -6544,123 +5901,70 @@
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="2"/>
-        <v>Low Growth Clean</v>
-      </c>
-      <c r="C12" t="str">
-        <v>low_growth_clean</v>
-      </c>
-      <c r="D12" s="2">
-        <f t="shared" si="0"/>
-        <v>0.92198577445123198</v>
-      </c>
-      <c r="E12" s="2">
-        <f t="shared" si="1"/>
-        <v>172.63357280995299</v>
-      </c>
-      <c r="F12" s="3">
-        <v>4.3768768088682908</v>
-      </c>
-      <c r="G12" s="5">
-        <f t="shared" si="5"/>
-        <v>5.2274474399100086</v>
-      </c>
-      <c r="H12" s="2">
-        <f t="shared" si="4"/>
-        <v>-120.55907571662162</v>
-      </c>
-      <c r="I12" s="2">
-        <f>G11-G12</f>
-        <v>2.6269452715440025</v>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="3"/>
+      <c r="H12" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" s="5">
+        <f>G3-G4</f>
+        <v>5.0595399552729816</v>
       </c>
       <c r="J12" s="2"/>
       <c r="R12" s="4"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="2"/>
-        <v>Low Growth Clean 400</v>
-      </c>
-      <c r="C13" t="str">
-        <v>low_growth_clean_400</v>
-      </c>
-      <c r="D13" s="2" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E13" s="2" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F13" s="3" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="G13" s="5" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H13" s="2" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="3"/>
+      <c r="H13" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="8">
+        <f>I12/I11</f>
+        <v>0.17032489070763449</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="R13" s="4"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="str">
-        <f t="shared" si="2"/>
-        <v>Low Growth Clean 500</v>
-      </c>
-      <c r="C14" t="str">
-        <v>low_growth_clean_500</v>
-      </c>
-      <c r="D14" s="2" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E14" s="2" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F14" s="3" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="G14" s="5" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H14" s="2" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="3"/>
+      <c r="H14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" s="5">
+        <f>G5-G3</f>
+        <v>40.545534618661009</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="R14" s="4"/>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
-      <c r="F15" s="3" t="e">
-        <v>#N/A</v>
+      <c r="F15" s="3"/>
+      <c r="H15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="5">
+        <f>I14-(G6-G4)</f>
+        <v>8.4182761960310017</v>
       </c>
       <c r="R15" s="4"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="3" t="e">
-        <v>#N/A</v>
+      <c r="F16" s="3"/>
+      <c r="H16" t="s">
+        <v>33</v>
+      </c>
+      <c r="I16" s="8">
+        <f>I15/I14</f>
+        <v>0.20762523605143204</v>
       </c>
       <c r="R16" s="4"/>
     </row>
@@ -6669,11 +5973,11 @@
       <c r="E17" s="2"/>
       <c r="F17" s="3"/>
       <c r="H17" t="s">
-        <v>33</v>
-      </c>
-      <c r="I17" s="5">
-        <f>G3</f>
-        <v>29.705229425086003</v>
+        <v>34</v>
+      </c>
+      <c r="I17" s="7">
+        <f>G5-G6</f>
+        <v>13.477816151303983</v>
       </c>
       <c r="R17" s="4"/>
     </row>
@@ -6681,75 +5985,33 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
-      <c r="H18" t="s">
-        <v>34</v>
-      </c>
-      <c r="I18" s="5">
-        <f>G3-G4</f>
-        <v>5.0595399552729816</v>
-      </c>
       <c r="R18" s="4"/>
     </row>
     <row r="19" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
-      <c r="H19" t="s">
-        <v>35</v>
-      </c>
-      <c r="I19" s="8">
-        <f>I18/I17</f>
-        <v>0.17032489070763449</v>
-      </c>
       <c r="R19" s="4"/>
     </row>
     <row r="20" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
-      <c r="H20" t="s">
-        <v>36</v>
-      </c>
-      <c r="I20" s="5">
-        <f>G7-G3</f>
-        <v>40.545534618661009</v>
-      </c>
     </row>
     <row r="21" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="3"/>
-      <c r="H21" t="s">
-        <v>37</v>
-      </c>
-      <c r="I21" s="5">
-        <f>I20-(G8-G4)</f>
-        <v>8.4182761960310017</v>
-      </c>
     </row>
     <row r="22" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="3"/>
-      <c r="H22" t="s">
-        <v>37</v>
-      </c>
-      <c r="I22" s="8">
-        <f>I21/I20</f>
-        <v>0.20762523605143204</v>
-      </c>
     </row>
     <row r="23" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
-      <c r="H23" t="s">
-        <v>38</v>
-      </c>
-      <c r="I23" s="7">
-        <f>G7-G8</f>
-        <v>13.477816151303983</v>
-      </c>
     </row>
     <row r="24" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D24" s="2"/>
@@ -6768,57 +6030,27 @@
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="3"/>
+      <c r="E27" s="1"/>
     </row>
     <row r="28" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="3"/>
+      <c r="E28" s="1"/>
     </row>
     <row r="29" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="3"/>
+      <c r="E29" s="1"/>
     </row>
     <row r="30" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="3"/>
+      <c r="E30" s="1"/>
     </row>
     <row r="31" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="3"/>
+      <c r="E31" s="1"/>
     </row>
     <row r="32" spans="4:18" x14ac:dyDescent="0.2">
       <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D33" s="2"/>
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D34" s="2"/>
-      <c r="E34" s="1"/>
-    </row>
-    <row r="35" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D35" s="2"/>
-      <c r="E35" s="1"/>
-    </row>
-    <row r="36" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D36" s="2"/>
-      <c r="E36" s="1"/>
-    </row>
-    <row r="37" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D37" s="2"/>
-      <c r="E37" s="1"/>
-    </row>
-    <row r="38" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D38" s="2"/>
-      <c r="E38" s="1"/>
+      <c r="E32" s="1"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L3:O18">
@@ -6833,12 +6065,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003E2EF3AF50F2594E8CFB88B65572827E" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a33f5ba277e803051ddec0c2f3ebdf97">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a92bd8f1-c682-480b-a293-fac44964c998" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb62609f8c3c2c61753a70ad7027dc26" ns2:_="">
     <xsd:import namespace="a92bd8f1-c682-480b-a293-fac44964c998"/>
@@ -7014,32 +6255,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8383D29D-B81E-419B-A632-579826696601}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A117057-420B-492F-A8C5-0D45FC583F79}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a92bd8f1-c682-480b-a293-fac44964c998"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8383D29D-B81E-419B-A632-579826696601}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a92bd8f1-c682-480b-a293-fac44964c998"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE72451-0000-473C-9BEF-3C3A5A240ABF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7057,14 +6297,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A117057-420B-492F-A8C5-0D45FC583F79}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" enabled="0" method="" siteId="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" removed="1"/>

</xml_diff>